<commit_message>
Fix: Notebook M1-M13 con codigo real explícito celda a celda y PDF con Índice General de 2 páginas
</commit_message>
<xml_diff>
--- a/04_Modelo_Excel/Valuacion_Aluar_Modelo_Oficial.xlsx
+++ b/04_Modelo_Excel/Valuacion_Aluar_Modelo_Oficial.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedea\Valuacion\valuacion-aluar-uncuyo\04_Modelo_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D30FA55F-6F1E-455E-8FBE-6F5541DB8478}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{409F0703-E3B5-40E9-8C73-52EE7135CF69}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A" sheetId="1" r:id="rId1"/>
@@ -6817,7 +6817,7 @@
         <v>211</v>
       </c>
       <c r="B80" s="66">
-        <f t="shared" ref="B80:G89" si="16">B30/B$2</f>
+        <f t="shared" ref="B80:G86" si="16">B30/B$2</f>
         <v>149756889.88311687</v>
       </c>
       <c r="C80" s="66">
@@ -8538,6 +8538,7 @@
   <sheetFormatPr baseColWidth="10" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="2" max="2" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="17.33203125" bestFit="1" customWidth="1"/>
     <col min="9" max="9" width="18.5546875" bestFit="1" customWidth="1"/>
     <col min="10" max="10" width="14.88671875" bestFit="1" customWidth="1"/>
   </cols>
@@ -9423,6 +9424,9 @@
       <c r="E43" s="92">
         <v>0.62016836374041573</v>
       </c>
+      <c r="F43">
+        <v>1584.2532379303639</v>
+      </c>
       <c r="I43" s="50" t="s">
         <v>287</v>
       </c>
@@ -9437,6 +9441,10 @@
       <c r="E44" s="94">
         <f>(E42/E43)-1</f>
         <v>0.2575117547292749</v>
+      </c>
+      <c r="F44">
+        <f>F43*E42</f>
+        <v>1235.51</v>
       </c>
       <c r="I44" s="50" t="s">
         <v>292</v>

</xml_diff>

<commit_message>
Corregir RR y WACC en fórmula del TV, unificar tickers de comparables, sacar generadores del repo y frases de IA
</commit_message>
<xml_diff>
--- a/04_Modelo_Excel/Valuacion_Aluar_Modelo_Oficial.xlsx
+++ b/04_Modelo_Excel/Valuacion_Aluar_Modelo_Oficial.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30228"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30326"/>
   <workbookPr defaultThemeVersion="202300"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\fedea\Valuacion\valuacion-aluar-uncuyo\04_Modelo_Excel\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3FA1EBBE-8E91-4FD0-AF10-B58BE9AB1A87}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{4E42299B-3F8C-4CBF-9074-568D86615AE8}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13176" firstSheet="1" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="A" sheetId="1" r:id="rId1"/>
@@ -7010,7 +7010,7 @@
         <v>211</v>
       </c>
       <c r="B80" s="66">
-        <f t="shared" ref="B80:G89" si="16">B30/B$2</f>
+        <f t="shared" ref="B80:G86" si="16">B30/B$2</f>
         <v>149756889.88311687</v>
       </c>
       <c r="C80" s="66">
@@ -8865,7 +8865,7 @@
       </c>
       <c r="J9" s="82">
         <f>J5+(J8*(J7-J5))+$J$21*J6</f>
-        <v>9.295115384748498E-2</v>
+        <v>9.1262123847484986E-2</v>
       </c>
       <c r="K9" s="106"/>
       <c r="L9" s="107"/>
@@ -8988,7 +8988,7 @@
       </c>
       <c r="J13" s="16">
         <f>J9*J12+J10*(1-J11)*(1-J12)</f>
-        <v>7.0637680200141537E-2</v>
+        <v>6.9501110582522438E-2</v>
       </c>
       <c r="K13" s="108"/>
       <c r="L13" s="109"/>
@@ -9162,7 +9162,7 @@
         <v>318</v>
       </c>
       <c r="J21" s="85">
-        <v>0.2</v>
+        <v>0.16170000000000001</v>
       </c>
     </row>
     <row r="22" spans="2:10" x14ac:dyDescent="0.3">
@@ -9439,19 +9439,19 @@
       </c>
       <c r="D32" s="86">
         <f>D31/(1+$J$13)</f>
-        <v>187471941.30255818</v>
+        <v>187671169.62549514</v>
       </c>
       <c r="E32" s="86">
         <f>E31/(1+$J$13)^2</f>
-        <v>164423849.73488352</v>
+        <v>164773505.19451872</v>
       </c>
       <c r="F32" s="86">
         <f>F31/(1+$J$13)^3</f>
-        <v>143600991.67967731</v>
+        <v>144059297.04735842</v>
       </c>
       <c r="G32" s="86">
         <f>G31/(1+$J$13)^4</f>
-        <v>124810065.91219366</v>
+        <v>125341459.90276912</v>
       </c>
     </row>
     <row r="33" spans="2:18" x14ac:dyDescent="0.3">
@@ -9460,7 +9460,7 @@
       </c>
       <c r="C33" s="86">
         <f>SUM(C32:G32)</f>
-        <v>562849853.66453946</v>
+        <v>564388436.80536819</v>
       </c>
       <c r="D33" s="54"/>
       <c r="E33" s="54"/>
@@ -9473,7 +9473,7 @@
       </c>
       <c r="E36" s="88">
         <f>C33</f>
-        <v>562849853.66453946</v>
+        <v>564388436.80536819</v>
       </c>
       <c r="I36" s="3" t="s">
         <v>324</v>
@@ -9507,7 +9507,7 @@
       </c>
       <c r="E37" s="88">
         <f>((G26+G27)*(1+$J$14))/($J$13-$J$14)/(1+$J$13)^4</f>
-        <v>2076783366.8168819</v>
+        <v>2133512502.0558231</v>
       </c>
       <c r="I37" s="3" t="s">
         <v>325</v>
@@ -9582,7 +9582,7 @@
       </c>
       <c r="E40" s="88">
         <f>E36+E37-E38+E39</f>
-        <v>2183633220.4814215</v>
+        <v>2241900938.8611913</v>
       </c>
       <c r="I40" s="3" t="s">
         <v>331</v>
@@ -9605,7 +9605,7 @@
       </c>
       <c r="E42" s="91">
         <f>E40/E41</f>
-        <v>0.77986900731479336</v>
+        <v>0.80067890673613973</v>
       </c>
       <c r="I42" s="47" t="s">
         <v>334</v>
@@ -9634,11 +9634,11 @@
       </c>
       <c r="E44" s="94">
         <f>(E42/E43)-1</f>
-        <v>0.2575117547292749</v>
+        <v>0.291066996560438</v>
       </c>
       <c r="F44">
         <f>F43*E42</f>
-        <v>1235.5100000000002</v>
+        <v>1268.4781505392734</v>
       </c>
       <c r="I44" s="50" t="s">
         <v>300</v>

</xml_diff>